<commit_message>
4:53 pm Thursday, 27 August 2026 (IST)
</commit_message>
<xml_diff>
--- a/My-Learning-Status/Spring.xlsx
+++ b/My-Learning-Status/Spring.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akum1255\Desktop\Office\2.My Technical Expertise\Final-RoadMap\FINAL\My-Learning-Status\New\New folder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/53cc78ed7981026d/Desktop/Home/Final/FINAL/My-Learning-Status/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE3C0C49-D0C2-4B6E-91BC-E4D4285E7FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{FE3C0C49-D0C2-4B6E-91BC-E4D4285E7FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F071915F-09FA-4F8B-B4C1-E9730E613400}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Spring-T" sheetId="5" r:id="rId1"/>
@@ -836,21 +836,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C786FBCE-7289-44E9-B8CC-7F9AF256655E}">
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="43.81640625" customWidth="1"/>
-    <col min="2" max="2" width="29.1796875" customWidth="1"/>
-    <col min="3" max="3" width="25.36328125" customWidth="1"/>
-    <col min="4" max="4" width="30.453125" customWidth="1"/>
-    <col min="5" max="5" width="34.453125" customWidth="1"/>
-    <col min="6" max="6" width="25.1796875" customWidth="1"/>
-    <col min="7" max="7" width="35.453125" customWidth="1"/>
-    <col min="8" max="8" width="28.1796875" customWidth="1"/>
-    <col min="9" max="9" width="31.1796875" customWidth="1"/>
-    <col min="10" max="10" width="14.90625" customWidth="1"/>
+    <col min="1" max="1" width="43.77734375" customWidth="1"/>
+    <col min="2" max="2" width="29.21875" customWidth="1"/>
+    <col min="3" max="3" width="25.33203125" customWidth="1"/>
+    <col min="4" max="4" width="30.44140625" customWidth="1"/>
+    <col min="5" max="5" width="34.44140625" customWidth="1"/>
+    <col min="6" max="6" width="25.21875" customWidth="1"/>
+    <col min="7" max="7" width="35.44140625" customWidth="1"/>
+    <col min="8" max="8" width="28.21875" customWidth="1"/>
+    <col min="9" max="9" width="31.21875" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -870,7 +870,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
         <v>85</v>
       </c>
@@ -890,7 +890,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
         <v>86</v>
       </c>
@@ -910,7 +910,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>87</v>
       </c>
@@ -930,7 +930,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
         <v>88</v>
       </c>
@@ -950,7 +950,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
         <v>89</v>
       </c>
@@ -970,7 +970,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
         <v>90</v>
       </c>
@@ -990,7 +990,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>91</v>
       </c>
@@ -1010,7 +1010,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
         <v>92</v>
       </c>
@@ -1030,7 +1030,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1044,7 +1044,7 @@
       <c r="K10" s="10"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="6"/>
       <c r="B11" s="7"/>
       <c r="C11" s="7" t="s">
@@ -1060,16 +1060,16 @@
         <v>93</v>
       </c>
     </row>
-    <row r="17" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="18" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="19" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="20" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="21" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="22" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="23" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="24" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="25" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="26" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="17" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="18" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="19" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="20" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="21" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="22" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="23" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="24" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="25" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="26" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1078,23 +1078,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0BF5F15-287A-4483-B4FE-40043117B605}">
   <dimension ref="A1:K22"/>
-  <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="12" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.1796875" style="13" customWidth="1"/>
-    <col min="2" max="2" width="46.81640625" style="14" customWidth="1"/>
-    <col min="3" max="3" width="5.7265625" style="14" customWidth="1"/>
-    <col min="4" max="4" width="2.1796875" style="14" customWidth="1"/>
+    <col min="1" max="1" width="5.21875" style="13" customWidth="1"/>
+    <col min="2" max="2" width="61.33203125" style="14" customWidth="1"/>
+    <col min="3" max="3" width="5.77734375" style="14" customWidth="1"/>
+    <col min="4" max="4" width="2.21875" style="14" customWidth="1"/>
     <col min="5" max="5" width="5" style="13" customWidth="1"/>
-    <col min="6" max="6" width="54" style="14" customWidth="1"/>
-    <col min="7" max="7" width="5.54296875" style="14" customWidth="1"/>
-    <col min="8" max="8" width="2.1796875" style="14" customWidth="1"/>
-    <col min="9" max="9" width="5.453125" style="13" customWidth="1"/>
-    <col min="10" max="10" width="46.26953125" style="14" customWidth="1"/>
-    <col min="11" max="11" width="5.7265625" style="14" customWidth="1"/>
-    <col min="12" max="16384" width="8.7265625" style="14"/>
+    <col min="6" max="6" width="61.109375" style="14" customWidth="1"/>
+    <col min="7" max="7" width="5.5546875" style="14" customWidth="1"/>
+    <col min="8" max="8" width="2.21875" style="14" customWidth="1"/>
+    <col min="9" max="9" width="5.44140625" style="13" customWidth="1"/>
+    <col min="10" max="10" width="67.21875" style="14" customWidth="1"/>
+    <col min="11" max="11" width="5.77734375" style="14" customWidth="1"/>
+    <col min="12" max="16384" width="8.77734375" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
         <v>33</v>
       </c>
@@ -1125,7 +1125,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="18">
         <v>1</v>
       </c>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="K2" s="20"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="18">
         <v>2</v>
       </c>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="K3" s="20"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="18">
         <v>3</v>
       </c>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="K4" s="20"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="18">
         <v>4</v>
       </c>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="K5" s="20"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="18">
         <v>5</v>
       </c>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="K6" s="20"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="18">
         <v>6</v>
       </c>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="K7" s="20"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="18">
         <v>7</v>
       </c>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="K8" s="20"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="18">
         <v>8</v>
       </c>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="K9" s="20"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="18">
         <v>9</v>
       </c>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="K10" s="20"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="18">
         <v>10</v>
       </c>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="K11" s="20"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="18"/>
       <c r="B12" s="20"/>
       <c r="C12" s="20"/>
@@ -1388,7 +1388,7 @@
       <c r="J12" s="20"/>
       <c r="K12" s="20"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="18">
         <v>11</v>
       </c>
@@ -1409,7 +1409,7 @@
       <c r="J13" s="20"/>
       <c r="K13" s="20"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="18">
         <v>12</v>
       </c>
@@ -1430,7 +1430,7 @@
       <c r="J14" s="20"/>
       <c r="K14" s="20"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="18">
         <v>13</v>
       </c>
@@ -1451,7 +1451,7 @@
       <c r="J15" s="20"/>
       <c r="K15" s="20"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="18">
         <v>14</v>
       </c>
@@ -1472,7 +1472,7 @@
       <c r="J16" s="20"/>
       <c r="K16" s="20"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="18">
         <v>15</v>
       </c>
@@ -1493,7 +1493,7 @@
       <c r="J17" s="20"/>
       <c r="K17" s="20"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="18">
         <v>16</v>
       </c>
@@ -1514,7 +1514,7 @@
       <c r="J18" s="20"/>
       <c r="K18" s="20"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="18">
         <v>17</v>
       </c>
@@ -1535,7 +1535,7 @@
       <c r="J19" s="20"/>
       <c r="K19" s="20"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="18">
         <v>18</v>
       </c>
@@ -1556,7 +1556,7 @@
       <c r="J20" s="20"/>
       <c r="K20" s="20"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="18">
         <v>19</v>
       </c>
@@ -1577,7 +1577,7 @@
       <c r="J21" s="20"/>
       <c r="K21" s="20"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="18">
         <v>20</v>
       </c>

</xml_diff>